<commit_message>
Add Local Business Sales Analysis project
</commit_message>
<xml_diff>
--- a/sales_summary.xlsx
+++ b/sales_summary.xlsx
@@ -10,10 +10,11 @@
     <sheet name="1_Total_Sales" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2_Best_Selling_Products" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="3_Category_wise_Sales" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4_Sales_Trend" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5_Top_Revenue_Products" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6_Quantity_Sold" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7_Recommendations" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="4a_Sales_Trend_Weekly" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="4b_Sales_Trend_Monthly" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="5_Top_Revenue_Products" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="6_Quantity_Sold" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="7_Recommendations" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -485,7 +486,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>523642.4999999999</v>
+        <v>382218.88</v>
       </c>
     </row>
     <row r="3">
@@ -495,7 +496,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>529910.8099999999</v>
+        <v>386831.38</v>
       </c>
     </row>
     <row r="4">
@@ -505,7 +506,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>6268.310000000003</v>
+        <v>4612.500000000002</v>
       </c>
     </row>
     <row r="5">
@@ -515,7 +516,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="6">
@@ -525,7 +526,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>5907</v>
+        <v>4358</v>
       </c>
     </row>
     <row r="7">
@@ -535,7 +536,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>261.82125</v>
+        <v>254.8125866666667</v>
       </c>
     </row>
     <row r="8">
@@ -556,7 +557,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>2025-01-03</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -568,7 +569,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -623,20 +624,20 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Wheat Flour 5kg</t>
+          <t>Potato 1kg</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>335</v>
+        <v>233</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>87281.63</v>
+        <v>7355.4</v>
       </c>
     </row>
     <row r="3">
@@ -649,89 +650,89 @@
         <v>2</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>294</v>
+        <v>202</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>11267.23</v>
+        <v>7678.23</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Milk 1L</t>
+          <t>Curd 500g</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>249</v>
+        <v>195</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>15483.32</v>
+        <v>7356.81</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Butter 100g</t>
+          <t>Salt 1kg</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>297</v>
+        <v>185</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>17127.83</v>
+        <v>4035.66</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Potato 1kg</t>
+          <t>Milk 1L</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>275</v>
+        <v>150</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>8802.940000000001</v>
+        <v>9313.91</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Salt 1kg</t>
+          <t>Rice 5kg</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>232</v>
+        <v>214</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>5070.57</v>
+        <v>68783.96000000001</v>
       </c>
     </row>
     <row r="8">
@@ -744,13 +745,13 @@
         <v>7</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>229</v>
+        <v>162</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>10956.11</v>
+        <v>7719.5</v>
       </c>
     </row>
     <row r="9">
@@ -763,51 +764,51 @@
         <v>8</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>228</v>
+        <v>159</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>9516.530000000001</v>
+        <v>6683.29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Rice 5kg</t>
+          <t>Wheat Flour 5kg</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>230</v>
+        <v>157</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>73534.74000000001</v>
+        <v>41384.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Curd 500g</t>
+          <t>Toor Dal 1kg</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>218</v>
+        <v>147</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8300.4</v>
+        <v>23992.72</v>
       </c>
     </row>
   </sheetData>
@@ -874,16 +875,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>160816.37</v>
+        <v>110168.46</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>565</v>
+        <v>371</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>172</v>
+        <v>123</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>30.71</v>
+        <v>28.82</v>
       </c>
     </row>
     <row r="3">
@@ -896,60 +897,60 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>52844.39</v>
+        <v>44066.84</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>344</v>
+        <v>285</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>118</v>
+        <v>89</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>10.09</v>
+        <v>11.53</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Beverages</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>48834.51</v>
+        <v>39489.64</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>929</v>
+        <v>421</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>316</v>
+        <v>129</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>9.33</v>
+        <v>10.33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>47408.01</v>
+        <v>30917.84</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>523</v>
+        <v>617</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>185</v>
+        <v>228</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>9.050000000000001</v>
+        <v>8.09</v>
       </c>
     </row>
     <row r="6">
@@ -962,16 +963,16 @@
         <v>5</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>35053.3</v>
+        <v>28209.47</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>461</v>
+        <v>371</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>164</v>
+        <v>130</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>6.69</v>
+        <v>7.38</v>
       </c>
     </row>
     <row r="7">
@@ -984,16 +985,16 @@
         <v>6</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>32838.9</v>
+        <v>26370.33</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>313</v>
+        <v>256</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>6.27</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="8">
@@ -1006,16 +1007,16 @@
         <v>7</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>29586.7</v>
+        <v>21716.92</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>797</v>
+        <v>594</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>261</v>
+        <v>207</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>5.65</v>
+        <v>5.68</v>
       </c>
     </row>
     <row r="9">
@@ -1028,16 +1029,16 @@
         <v>8</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>28922.04</v>
+        <v>18632.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>301</v>
+        <v>198</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>5.52</v>
+        <v>4.87</v>
       </c>
     </row>
     <row r="10">
@@ -1050,60 +1051,60 @@
         <v>9</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>26287.9</v>
+        <v>17038.37</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>184</v>
+        <v>118</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>5.02</v>
+        <v>4.46</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Snacks</t>
+          <t>Spices</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>17219.11</v>
+        <v>13665.56</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>333</v>
+        <v>255</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>121</v>
+        <v>88</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>3.29</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Spices</t>
+          <t>Snacks</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>16791.19</v>
+        <v>12372.68</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>315</v>
+        <v>244</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>3.21</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="13">
@@ -1116,16 +1117,16 @@
         <v>12</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>16026.68</v>
+        <v>11755.16</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>461</v>
+        <v>347</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>170</v>
+        <v>132</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>3.06</v>
+        <v>3.08</v>
       </c>
     </row>
     <row r="14">
@@ -1138,16 +1139,16 @@
         <v>13</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>8487.219999999999</v>
+        <v>5778.35</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>212</v>
+        <v>144</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>1.62</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="15">
@@ -1160,16 +1161,16 @@
         <v>14</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>2526.18</v>
+        <v>2036.76</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>169</v>
+        <v>137</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.48</v>
+        <v>0.53</v>
       </c>
     </row>
   </sheetData>
@@ -1183,365 +1184,375 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Year_Month</t>
+          <t>Week_No</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Week_Start</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Week_End</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Total_Sales</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Change_%_vs_Previous_Month</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>3_Month_Moving_Avg</t>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Avg_Daily_Sales</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Change_%_vs_Previous_Week</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2025-01</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>22649.98</v>
-      </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr"/>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>41848.61</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>5978.37</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2025-02</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>24223.07</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>6.95</v>
-      </c>
-      <c r="D3" s="4" t="inlineStr"/>
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>34867.8</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>4981.11</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>-16.68</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2025-03</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>33893.66</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>39.92</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>26922.24</v>
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>30597.58</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>4371.08</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>-12.25</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>2025-04</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>24704.29</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>-27.11</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>27607.01</v>
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>40638.3</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>5805.47</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>32.82</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2025-05</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>22981.8</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>-6.97</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>27193.25</v>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>30033.2</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>4290.46</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>-26.1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>2025-06</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>19064.14</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>-17.05</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>22250.08</v>
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>26988.3</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>3855.47</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>-10.14</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>20446.92</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>7.25</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>20830.95</v>
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>27353.46</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>3907.64</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>1.35</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>22979.39</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>12.39</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>20830.15</v>
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>28167.71</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>4023.96</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>2.98</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>18273.91</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>-20.48</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>20566.74</v>
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>40955.92</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>5850.85</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>45.4</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>29490.87</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>61.38</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>23581.39</v>
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>34088.71</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>4869.82</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>-16.77</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>26945.73</v>
-      </c>
-      <c r="C12" s="3" t="n">
-        <v>-8.630000000000001</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>24903.5</v>
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>32452.66</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>4636.09</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>-4.8</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>29132.67</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>8.119999999999999</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>28523.09</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>31191.24</v>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>7.07</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>29089.88</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>28705.26</v>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>-7.97</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>29676.39</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>22324.95</v>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>-22.23</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>27407.15</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>25205.63</v>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>25411.95</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>25581.66</v>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>24370.75</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>15962.93</v>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>-37.6</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>22250.07</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>29828.52</v>
-      </c>
-      <c r="C20" s="3" t="n">
-        <v>86.86</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>23791.04</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>20838.62</v>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>-30.14</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>22210.02</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n">
-        <v>29217.26</v>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>40.21</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>26628.13</v>
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>14226.63</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>4742.21</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>2.29</v>
       </c>
     </row>
   </sheetData>
@@ -1550,6 +1561,109 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Year_Month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Sales</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Avg_Daily_Sales</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Change_%_vs_Previous_Month</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>150049.91</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>5174.13</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>135916</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>4384.39</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>-15.26</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>96252.97</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>4812.65</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>9.77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1595,96 +1709,96 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Wheat Flour 5kg</t>
+          <t>Rice 5kg</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>87281.63</v>
+        <v>68783.96000000001</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>16.67</v>
+        <v>18</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>16.67</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Rice 5kg</t>
+          <t>Wheat Flour 5kg</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>73534.74000000001</v>
+        <v>41384.5</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>14.04</v>
+        <v>10.83</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>30.71</v>
+        <v>28.82</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Moong Dal 1kg</t>
+          <t>Toor Dal 1kg</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>26568.98</v>
+        <v>23992.72</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>5.07</v>
+        <v>6.28</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>35.78</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Sunflower Oil 1L</t>
+          <t>Moong Dal 1kg</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>26287.9</v>
+        <v>20074.12</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>5.02</v>
+        <v>5.25</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>40.81</v>
+        <v>40.35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Toor Dal 1kg</t>
+          <t>Tea 250g</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>26275.41</v>
+        <v>18424.52</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>5.02</v>
+        <v>4.82</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>45.82</v>
+        <v>45.17</v>
       </c>
     </row>
     <row r="7">
@@ -1697,89 +1811,89 @@
         <v>6</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>23432.14</v>
+        <v>18217.5</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>4.47</v>
+        <v>4.77</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>50.3</v>
+        <v>49.94</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Tea 250g</t>
+          <t>Sunflower Oil 1L</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>22589.25</v>
+        <v>17038.37</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>4.31</v>
+        <v>4.46</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>54.61</v>
+        <v>54.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Detergent 1kg</t>
+          <t>Shampoo 180ml</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>17697.35</v>
+        <v>14758.39</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>3.38</v>
+        <v>3.86</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>57.99</v>
+        <v>58.26</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Butter 100g</t>
+          <t>Coffee 100g</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>17127.83</v>
+        <v>14684.92</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3.27</v>
+        <v>3.84</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>61.26</v>
+        <v>62.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Shampoo 180ml</t>
+          <t>Detergent 1kg</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>16942.21</v>
+        <v>9609.66</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>3.24</v>
+        <v>2.51</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>64.5</v>
+        <v>64.61</v>
       </c>
     </row>
   </sheetData>
@@ -1787,7 +1901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1827,33 +1941,33 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Wheat Flour 5kg</t>
+          <t>Potato 1kg</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>335</v>
+        <v>233</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>5.67</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Butter 100g</t>
+          <t>Rice 5kg</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>297</v>
+        <v>214</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>5.03</v>
+        <v>4.91</v>
       </c>
     </row>
     <row r="4">
@@ -1866,218 +1980,218 @@
         <v>3</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>294</v>
+        <v>202</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>4.98</v>
+        <v>4.64</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Potato 1kg</t>
+          <t>Curd 500g</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>275</v>
+        <v>195</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>4.66</v>
+        <v>4.47</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Milk 1L</t>
+          <t>Salt 1kg</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>249</v>
+        <v>185</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>4.22</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Salt 1kg</t>
+          <t>Sugar 1kg</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>232</v>
+        <v>162</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>3.93</v>
+        <v>3.72</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Rice 5kg</t>
+          <t>Tomato 1kg</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>230</v>
+        <v>159</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>3.89</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Sugar 1kg</t>
+          <t>Wheat Flour 5kg</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>229</v>
+        <v>157</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>3.88</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Tomato 1kg</t>
+          <t>Milk 1L</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>228</v>
+        <v>150</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3.86</v>
+        <v>3.44</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Curd 500g</t>
+          <t>Toor Dal 1kg</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>218</v>
+        <v>147</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>3.69</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Bread</t>
+          <t>Tea 250g</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
         <v>11</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>212</v>
+        <v>147</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>3.59</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Cold Drink 750ml</t>
+          <t>Eggs 6 Pack</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
         <v>12</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>197</v>
+        <v>145</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3.34</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Toothpaste</t>
+          <t>Bread</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
         <v>13</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>191</v>
+        <v>144</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>3.23</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Sunflower Oil 1L</t>
+          <t>Cold Drink 750ml</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
         <v>14</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>184</v>
+        <v>142</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3.11</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Moong Dal 1kg</t>
+          <t>Chilli Powder 200g</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
         <v>15</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>184</v>
+        <v>141</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>3.11</v>
+        <v>3.24</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Tea 250g</t>
+          <t>Moong Dal 1kg</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
         <v>16</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>181</v>
+        <v>138</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>3.06</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="18">
@@ -2090,218 +2204,218 @@
         <v>17</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>169</v>
+        <v>137</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>2.86</v>
+        <v>3.14</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Biscuits Pack</t>
+          <t>Banana Dozen</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
         <v>18</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>169</v>
+        <v>135</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>2.86</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Detergent 1kg</t>
+          <t>Biscuits Pack</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
         <v>19</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>169</v>
+        <v>133</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>2.86</v>
+        <v>3.05</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Chilli Powder 200g</t>
+          <t>Coffee 100g</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
         <v>20</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>166</v>
+        <v>132</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>2.81</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Eggs 6 Pack</t>
+          <t>Toothpaste</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
         <v>21</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>165</v>
+        <v>131</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>2.79</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Peanuts 500g</t>
+          <t>Butter 100g</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
         <v>22</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>164</v>
+        <v>127</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.78</v>
+        <v>2.91</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Toor Dal 1kg</t>
+          <t>Apples 1kg</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
         <v>23</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>2.71</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Banana Dozen</t>
+          <t>Bath Soap</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
         <v>24</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>157</v>
+        <v>121</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>2.66</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Apples 1kg</t>
+          <t>Shampoo 180ml</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
         <v>25</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>156</v>
+        <v>119</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>2.64</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Turmeric Powder 200g</t>
+          <t>Sunflower Oil 1L</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
         <v>26</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>2.52</v>
+        <v>2.71</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Coffee 100g</t>
+          <t>Turmeric Powder 200g</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
         <v>27</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>145</v>
+        <v>114</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>2.45</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Shampoo 180ml</t>
+          <t>Peanuts 500g</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
         <v>28</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>136</v>
+        <v>111</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>2.3</v>
+        <v>2.55</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Bath Soap</t>
+          <t>Dishwash Liquid</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
         <v>29</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>2.27</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Dishwash Liquid</t>
+          <t>Detergent 1kg</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
         <v>30</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>132</v>
+        <v>91</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>2.23</v>
+        <v>2.09</v>
       </c>
     </row>
   </sheetData>
@@ -2309,7 +2423,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2331,49 +2445,49 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>1. Keep the top revenue products always in stock: Wheat Flour 5kg, Rice 5kg, Moong Dal 1kg, Sunflower Oil 1L, Toor Dal 1kg.</t>
+          <t>1. Keep the top revenue products always in stock: Rice 5kg, Wheat Flour 5kg, Toor Dal 1kg, Moong Dal 1kg, Tea 250g.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>2. Grains is the strongest category (30.7% of sales); protect its supply and pricing.</t>
+          <t>2. Grains is the strongest category (28.8% of sales); protect its supply and pricing.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>3. Increase stock before Sunday and weekends; keep lower stock on Thursday.</t>
+          <t>3. Increase stock before Monday (highest average daily sales); keep lower stock on Tuesday.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>4. Offer bundle deals or discounts on slow products: Turmeric Powder 200g, Salt 1kg, Bath Soap, Biscuits Pack, Instant Noodles.</t>
+          <t>4. Offer bundle deals or discounts on slow products: Turmeric Powder 200g, Bath Soap, Salt 1kg, Biscuits Pack, Instant Noodles.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>5. Plan extra stock for the best month (2025-03) and reduce orders in the weakest month (2026-06).</t>
+          <t>5. Plan extra stock for strong weeks like Week 1 (2026-07-03 to 2026-07-09) and reduce orders in weak weeks like Week 6.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>6. Walk-in customers give 72.4% of sales; start loyalty offers to make them regular.</t>
+          <t>6. Walk-in customers give 73.3% of sales; start loyalty offers to make them regular.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>7. UPI is the most used payment method (49.5%); promote digital payments.</t>
+          <t>7. UPI is the most used payment method (46.9%); promote digital payments.</t>
         </is>
       </c>
     </row>

</xml_diff>